<commit_message>
Script unificado otimizado sem erros de terminal do Yahoo
</commit_message>
<xml_diff>
--- a/fiis_b3.xlsx
+++ b/fiis_b3.xlsx
@@ -697,7 +697,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -1089,7 +1089,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -2167,7 +2167,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2265,7 +2265,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2363,7 +2363,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2853,7 +2853,7 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -3343,7 +3343,7 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
@@ -3833,7 +3833,7 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
@@ -4225,7 +4225,7 @@
         </is>
       </c>
       <c r="P39" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
         </is>
       </c>
       <c r="P40" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
@@ -4617,7 +4617,7 @@
         </is>
       </c>
       <c r="P43" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
@@ -4715,7 +4715,7 @@
         </is>
       </c>
       <c r="P44" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
@@ -6185,7 +6185,7 @@
         </is>
       </c>
       <c r="P59" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
@@ -6283,7 +6283,7 @@
         </is>
       </c>
       <c r="P60" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
@@ -6479,7 +6479,7 @@
         </is>
       </c>
       <c r="P62" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q62" t="inlineStr">
         <is>
@@ -6675,7 +6675,7 @@
         </is>
       </c>
       <c r="P64" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
@@ -6773,7 +6773,7 @@
         </is>
       </c>
       <c r="P65" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q65" t="inlineStr">
         <is>
@@ -7459,7 +7459,7 @@
         </is>
       </c>
       <c r="P72" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q72" t="inlineStr">
         <is>
@@ -7851,7 +7851,7 @@
         </is>
       </c>
       <c r="P76" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
@@ -8733,7 +8733,7 @@
         </is>
       </c>
       <c r="P85" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q85" t="inlineStr">
         <is>
@@ -8831,7 +8831,7 @@
         </is>
       </c>
       <c r="P86" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q86" t="inlineStr">
         <is>
@@ -9223,7 +9223,7 @@
         </is>
       </c>
       <c r="P90" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q90" t="inlineStr">
         <is>
@@ -9713,7 +9713,7 @@
         </is>
       </c>
       <c r="P95" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q95" t="inlineStr">
         <is>
@@ -10007,7 +10007,7 @@
         </is>
       </c>
       <c r="P98" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q98" t="inlineStr">
         <is>
@@ -10497,7 +10497,7 @@
         </is>
       </c>
       <c r="P103" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="Q103" t="inlineStr">
         <is>
@@ -10791,7 +10791,7 @@
         </is>
       </c>
       <c r="P106" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q106" t="inlineStr">
         <is>
@@ -10889,7 +10889,7 @@
         </is>
       </c>
       <c r="P107" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q107" t="inlineStr">
         <is>
@@ -11183,7 +11183,7 @@
         </is>
       </c>
       <c r="P110" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q110" t="inlineStr">
         <is>
@@ -11477,7 +11477,7 @@
         </is>
       </c>
       <c r="P113" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q113" t="inlineStr">
         <is>
@@ -11575,7 +11575,7 @@
         </is>
       </c>
       <c r="P114" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q114" t="inlineStr">
         <is>
@@ -12457,7 +12457,7 @@
         </is>
       </c>
       <c r="P123" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q123" t="inlineStr">
         <is>
@@ -12751,7 +12751,7 @@
         </is>
       </c>
       <c r="P126" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q126" t="inlineStr">
         <is>
@@ -12947,7 +12947,7 @@
         </is>
       </c>
       <c r="P128" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q128" t="inlineStr">
         <is>
@@ -13927,7 +13927,7 @@
         </is>
       </c>
       <c r="P138" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q138" t="inlineStr">
         <is>
@@ -14221,7 +14221,7 @@
         </is>
       </c>
       <c r="P141" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q141" t="inlineStr">
         <is>
@@ -14319,7 +14319,7 @@
         </is>
       </c>
       <c r="P142" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q142" t="inlineStr">
         <is>
@@ -14515,7 +14515,7 @@
         </is>
       </c>
       <c r="P144" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q144" t="inlineStr">
         <is>
@@ -14711,7 +14711,7 @@
         </is>
       </c>
       <c r="P146" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q146" t="inlineStr">
         <is>
@@ -14907,7 +14907,7 @@
         </is>
       </c>
       <c r="P148" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q148" t="inlineStr">
         <is>
@@ -15005,7 +15005,7 @@
         </is>
       </c>
       <c r="P149" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q149" t="inlineStr">
         <is>
@@ -15103,7 +15103,7 @@
         </is>
       </c>
       <c r="P150" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q150" t="inlineStr">
         <is>
@@ -15201,7 +15201,7 @@
         </is>
       </c>
       <c r="P151" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q151" t="inlineStr">
         <is>
@@ -15691,7 +15691,7 @@
         </is>
       </c>
       <c r="P156" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q156" t="inlineStr">
         <is>
@@ -15789,7 +15789,7 @@
         </is>
       </c>
       <c r="P157" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q157" t="inlineStr">
         <is>
@@ -15887,7 +15887,7 @@
         </is>
       </c>
       <c r="P158" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q158" t="inlineStr">
         <is>
@@ -15985,7 +15985,7 @@
         </is>
       </c>
       <c r="P159" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q159" t="inlineStr">
         <is>
@@ -16377,7 +16377,7 @@
         </is>
       </c>
       <c r="P163" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q163" t="inlineStr">
         <is>
@@ -16573,7 +16573,7 @@
         </is>
       </c>
       <c r="P165" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q165" t="inlineStr">
         <is>
@@ -16671,7 +16671,7 @@
         </is>
       </c>
       <c r="P166" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q166" t="inlineStr">
         <is>
@@ -17847,7 +17847,7 @@
         </is>
       </c>
       <c r="P178" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="Q178" t="inlineStr">
         <is>
@@ -18533,7 +18533,7 @@
         </is>
       </c>
       <c r="P185" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q185" t="inlineStr">
         <is>
@@ -18729,7 +18729,7 @@
         </is>
       </c>
       <c r="P187" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q187" t="inlineStr">
         <is>
@@ -19219,7 +19219,7 @@
         </is>
       </c>
       <c r="P192" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q192" t="inlineStr">
         <is>
@@ -19709,7 +19709,7 @@
         </is>
       </c>
       <c r="P197" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q197" t="inlineStr">
         <is>
@@ -19807,7 +19807,7 @@
         </is>
       </c>
       <c r="P198" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q198" t="inlineStr">
         <is>
@@ -20003,7 +20003,7 @@
         </is>
       </c>
       <c r="P200" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q200" t="inlineStr">
         <is>
@@ -20297,7 +20297,7 @@
         </is>
       </c>
       <c r="P203" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q203" t="inlineStr">
         <is>
@@ -20395,7 +20395,7 @@
         </is>
       </c>
       <c r="P204" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q204" t="inlineStr">
         <is>
@@ -20493,7 +20493,7 @@
         </is>
       </c>
       <c r="P205" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q205" t="inlineStr">
         <is>
@@ -20787,7 +20787,7 @@
         </is>
       </c>
       <c r="P208" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q208" t="inlineStr">
         <is>
@@ -20885,7 +20885,7 @@
         </is>
       </c>
       <c r="P209" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q209" t="inlineStr">
         <is>
@@ -20983,7 +20983,7 @@
         </is>
       </c>
       <c r="P210" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q210" t="inlineStr">
         <is>
@@ -21081,7 +21081,7 @@
         </is>
       </c>
       <c r="P211" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q211" t="inlineStr">
         <is>
@@ -21473,7 +21473,7 @@
         </is>
       </c>
       <c r="P215" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q215" t="inlineStr">
         <is>
@@ -21767,7 +21767,7 @@
         </is>
       </c>
       <c r="P218" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q218" t="inlineStr">
         <is>
@@ -21865,7 +21865,7 @@
         </is>
       </c>
       <c r="P219" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q219" t="inlineStr">
         <is>
@@ -21963,7 +21963,7 @@
         </is>
       </c>
       <c r="P220" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q220" t="inlineStr">
         <is>
@@ -22453,7 +22453,7 @@
         </is>
       </c>
       <c r="P225" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q225" t="inlineStr">
         <is>
@@ -22649,7 +22649,7 @@
         </is>
       </c>
       <c r="P227" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q227" t="inlineStr">
         <is>
@@ -22845,7 +22845,7 @@
         </is>
       </c>
       <c r="P229" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q229" t="inlineStr">
         <is>
@@ -24315,7 +24315,7 @@
         </is>
       </c>
       <c r="P244" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q244" t="inlineStr">
         <is>
@@ -24413,7 +24413,7 @@
         </is>
       </c>
       <c r="P245" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q245" t="inlineStr">
         <is>
@@ -25687,7 +25687,7 @@
         </is>
       </c>
       <c r="P258" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q258" t="inlineStr">
         <is>
@@ -26177,7 +26177,7 @@
         </is>
       </c>
       <c r="P263" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q263" t="inlineStr">
         <is>
@@ -26667,7 +26667,7 @@
         </is>
       </c>
       <c r="P268" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q268" t="inlineStr">
         <is>
@@ -27157,7 +27157,7 @@
         </is>
       </c>
       <c r="P273" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q273" t="inlineStr">
         <is>
@@ -27353,7 +27353,7 @@
         </is>
       </c>
       <c r="P275" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q275" t="inlineStr">
         <is>
@@ -27451,7 +27451,7 @@
         </is>
       </c>
       <c r="P276" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="Q276" t="inlineStr">
         <is>
@@ -27647,7 +27647,7 @@
         </is>
       </c>
       <c r="P278" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="Q278" t="inlineStr">
         <is>
@@ -27745,7 +27745,7 @@
         </is>
       </c>
       <c r="P279" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q279" t="inlineStr">
         <is>
@@ -29999,7 +29999,7 @@
         </is>
       </c>
       <c r="P302" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q302" t="inlineStr">
         <is>
@@ -30391,7 +30391,7 @@
         </is>
       </c>
       <c r="P306" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q306" t="inlineStr">
         <is>
@@ -30489,7 +30489,7 @@
         </is>
       </c>
       <c r="P307" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q307" t="inlineStr">
         <is>
@@ -30587,7 +30587,7 @@
         </is>
       </c>
       <c r="P308" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q308" t="inlineStr">
         <is>
@@ -31371,7 +31371,7 @@
         </is>
       </c>
       <c r="P316" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q316" t="inlineStr">
         <is>
@@ -32449,7 +32449,7 @@
         </is>
       </c>
       <c r="P327" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q327" t="inlineStr">
         <is>
@@ -32743,7 +32743,7 @@
         </is>
       </c>
       <c r="P330" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q330" t="inlineStr">
         <is>
@@ -33037,7 +33037,7 @@
         </is>
       </c>
       <c r="P333" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q333" t="inlineStr">
         <is>
@@ -33135,7 +33135,7 @@
         </is>
       </c>
       <c r="P334" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q334" t="inlineStr">
         <is>
@@ -33429,7 +33429,7 @@
         </is>
       </c>
       <c r="P337" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q337" t="inlineStr">
         <is>
@@ -33527,7 +33527,7 @@
         </is>
       </c>
       <c r="P338" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q338" t="inlineStr">
         <is>
@@ -34605,7 +34605,7 @@
         </is>
       </c>
       <c r="P349" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="Q349" t="inlineStr">
         <is>
@@ -35095,7 +35095,7 @@
         </is>
       </c>
       <c r="P354" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q354" t="inlineStr">
         <is>
@@ -35291,7 +35291,7 @@
         </is>
       </c>
       <c r="P356" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q356" t="inlineStr">
         <is>
@@ -35683,7 +35683,7 @@
         </is>
       </c>
       <c r="P360" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q360" t="inlineStr">
         <is>
@@ -36075,7 +36075,7 @@
         </is>
       </c>
       <c r="P364" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q364" t="inlineStr">
         <is>
@@ -36369,7 +36369,7 @@
         </is>
       </c>
       <c r="P367" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q367" t="inlineStr">
         <is>
@@ -36957,7 +36957,7 @@
         </is>
       </c>
       <c r="P373" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q373" t="inlineStr">
         <is>
@@ -37153,7 +37153,7 @@
         </is>
       </c>
       <c r="P375" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q375" t="inlineStr">
         <is>
@@ -37251,7 +37251,7 @@
         </is>
       </c>
       <c r="P376" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q376" t="inlineStr">
         <is>
@@ -37349,7 +37349,7 @@
         </is>
       </c>
       <c r="P377" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q377" t="inlineStr">
         <is>
@@ -37447,7 +37447,7 @@
         </is>
       </c>
       <c r="P378" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q378" t="inlineStr">
         <is>
@@ -38427,7 +38427,7 @@
         </is>
       </c>
       <c r="P388" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q388" t="inlineStr">
         <is>
@@ -38525,7 +38525,7 @@
         </is>
       </c>
       <c r="P389" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q389" t="inlineStr">
         <is>
@@ -38819,7 +38819,7 @@
         </is>
       </c>
       <c r="P392" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q392" t="inlineStr">
         <is>
@@ -39309,7 +39309,7 @@
         </is>
       </c>
       <c r="P397" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q397" t="inlineStr">
         <is>
@@ -39603,7 +39603,7 @@
         </is>
       </c>
       <c r="P400" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q400" t="inlineStr">
         <is>
@@ -39701,7 +39701,7 @@
         </is>
       </c>
       <c r="P401" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q401" t="inlineStr">
         <is>
@@ -39799,7 +39799,7 @@
         </is>
       </c>
       <c r="P402" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="Q402" t="inlineStr">
         <is>
@@ -40093,7 +40093,7 @@
         </is>
       </c>
       <c r="P405" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q405" t="inlineStr">
         <is>
@@ -40191,7 +40191,7 @@
         </is>
       </c>
       <c r="P406" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q406" t="inlineStr">
         <is>
@@ -40289,7 +40289,7 @@
         </is>
       </c>
       <c r="P407" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q407" t="inlineStr">
         <is>
@@ -40583,7 +40583,7 @@
         </is>
       </c>
       <c r="P410" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q410" t="inlineStr">
         <is>
@@ -40681,7 +40681,7 @@
         </is>
       </c>
       <c r="P411" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q411" t="inlineStr">
         <is>
@@ -40779,7 +40779,7 @@
         </is>
       </c>
       <c r="P412" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q412" t="inlineStr">
         <is>
@@ -41073,7 +41073,7 @@
         </is>
       </c>
       <c r="P415" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q415" t="inlineStr">
         <is>
@@ -41955,7 +41955,7 @@
         </is>
       </c>
       <c r="P424" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q424" t="inlineStr">
         <is>
@@ -42151,7 +42151,7 @@
         </is>
       </c>
       <c r="P426" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q426" t="inlineStr">
         <is>
@@ -42543,7 +42543,7 @@
         </is>
       </c>
       <c r="P430" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q430" t="inlineStr">
         <is>
@@ -42935,7 +42935,7 @@
         </is>
       </c>
       <c r="P434" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q434" t="inlineStr">
         <is>
@@ -43033,7 +43033,7 @@
         </is>
       </c>
       <c r="P435" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q435" t="inlineStr">
         <is>
@@ -43523,7 +43523,7 @@
         </is>
       </c>
       <c r="P440" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q440" t="inlineStr">
         <is>
@@ -44895,7 +44895,7 @@
         </is>
       </c>
       <c r="P454" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q454" t="inlineStr">
         <is>
@@ -45091,7 +45091,7 @@
         </is>
       </c>
       <c r="P456" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q456" t="inlineStr">
         <is>
@@ -45189,7 +45189,7 @@
         </is>
       </c>
       <c r="P457" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q457" t="inlineStr">
         <is>
@@ -45287,7 +45287,7 @@
         </is>
       </c>
       <c r="P458" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q458" t="inlineStr">
         <is>
@@ -45875,7 +45875,7 @@
         </is>
       </c>
       <c r="P464" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q464" t="inlineStr">
         <is>
@@ -47639,7 +47639,7 @@
         </is>
       </c>
       <c r="P482" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q482" t="inlineStr">
         <is>
@@ -48227,7 +48227,7 @@
         </is>
       </c>
       <c r="P488" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q488" t="inlineStr">
         <is>
@@ -48325,7 +48325,7 @@
         </is>
       </c>
       <c r="P489" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="Q489" t="inlineStr">
         <is>
@@ -49207,7 +49207,7 @@
         </is>
       </c>
       <c r="P498" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q498" t="inlineStr">
         <is>
@@ -49403,7 +49403,7 @@
         </is>
       </c>
       <c r="P500" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q500" t="inlineStr">
         <is>
@@ -50285,7 +50285,7 @@
         </is>
       </c>
       <c r="P509" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q509" t="inlineStr">
         <is>
@@ -50677,7 +50677,7 @@
         </is>
       </c>
       <c r="P513" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q513" t="inlineStr">
         <is>
@@ -51069,7 +51069,7 @@
         </is>
       </c>
       <c r="P517" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q517" t="inlineStr">
         <is>
@@ -51167,7 +51167,7 @@
         </is>
       </c>
       <c r="P518" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q518" t="inlineStr">
         <is>
@@ -51559,7 +51559,7 @@
         </is>
       </c>
       <c r="P522" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q522" t="inlineStr">
         <is>
@@ -51657,7 +51657,7 @@
         </is>
       </c>
       <c r="P523" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q523" t="inlineStr">
         <is>
@@ -51755,7 +51755,7 @@
         </is>
       </c>
       <c r="P524" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="Q524" t="inlineStr">
         <is>
@@ -52147,7 +52147,7 @@
         </is>
       </c>
       <c r="P528" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q528" t="inlineStr">
         <is>
@@ -52343,7 +52343,7 @@
         </is>
       </c>
       <c r="P530" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q530" t="inlineStr">
         <is>
@@ -52637,7 +52637,7 @@
         </is>
       </c>
       <c r="P533" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q533" t="inlineStr">
         <is>
@@ -53029,7 +53029,7 @@
         </is>
       </c>
       <c r="P537" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q537" t="inlineStr">
         <is>
@@ -53617,7 +53617,7 @@
         </is>
       </c>
       <c r="P543" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q543" t="inlineStr">
         <is>
@@ -53813,7 +53813,7 @@
         </is>
       </c>
       <c r="P545" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q545" t="inlineStr">
         <is>
@@ -54107,7 +54107,7 @@
         </is>
       </c>
       <c r="P548" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q548" t="inlineStr">
         <is>
@@ -54205,7 +54205,7 @@
         </is>
       </c>
       <c r="P549" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q549" t="inlineStr">
         <is>
@@ -54303,7 +54303,7 @@
         </is>
       </c>
       <c r="P550" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q550" t="inlineStr">
         <is>
@@ -54401,7 +54401,7 @@
         </is>
       </c>
       <c r="P551" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q551" t="inlineStr">
         <is>
@@ -54499,7 +54499,7 @@
         </is>
       </c>
       <c r="P552" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q552" t="inlineStr">
         <is>
@@ -54597,7 +54597,7 @@
         </is>
       </c>
       <c r="P553" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q553" t="inlineStr">
         <is>
@@ -54793,7 +54793,7 @@
         </is>
       </c>
       <c r="P555" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q555" t="inlineStr">
         <is>

</xml_diff>